<commit_message>
completeTitle for cvAcademicTitle criterion
</commit_message>
<xml_diff>
--- a/criterion_property_definitions.xlsx
+++ b/criterion_property_definitions.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\configuration\master-data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BEF0077-2C24-42D9-BD93-6940AED9DFEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2EA08C86-2099-4477-8DAF-87FA7BC27135}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="390" yWindow="390" windowWidth="48570" windowHeight="13875" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="16470" yWindow="2160" windowWidth="48570" windowHeight="13875" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="criterion_property" sheetId="4" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1838" uniqueCount="459">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1839" uniqueCount="460">
   <si>
     <t>property</t>
   </si>
@@ -1405,6 +1405,9 @@
   </si>
   <si>
     <t>staff.personParticulars.cvAcademicTitle</t>
+  </si>
+  <si>
+    <t>completeTitle</t>
   </si>
 </sst>
 </file>
@@ -2373,6 +2376,9 @@
       <c r="C28" t="s">
         <v>15</v>
       </c>
+      <c r="H28" t="s">
+        <v>459</v>
+      </c>
       <c r="L28" t="s">
         <v>458</v>
       </c>

</xml_diff>

<commit_message>
drop LIKE support for normalizedName criterions
</commit_message>
<xml_diff>
--- a/criterion_property_definitions.xlsx
+++ b/criterion_property_definitions.xlsx
@@ -1372,7 +1372,7 @@
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>EQ, NE, GT, GE, LT, LE, LIKE, ILIKE</t>
+          <t>EQ, NE, GT, GE, LT, LE</t>
         </is>
       </c>
     </row>
@@ -1426,7 +1426,7 @@
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>EQ, NE, GT, GE, LT, LE, LIKE, ILIKE</t>
+          <t>EQ, NE, GT, GE, LT, LE</t>
         </is>
       </c>
     </row>
@@ -1512,7 +1512,7 @@
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>EQ, NE, GT, GE, LT, LE, LIKE, ILIKE</t>
+          <t>EQ, NE, GT, GE, LT, LE</t>
         </is>
       </c>
     </row>
@@ -4767,7 +4767,7 @@
       </c>
       <c r="M137" t="inlineStr">
         <is>
-          <t>EQ, NE, LIKE, ILIKE</t>
+          <t>EQ, NE</t>
         </is>
       </c>
     </row>
@@ -4821,7 +4821,7 @@
       </c>
       <c r="M139" t="inlineStr">
         <is>
-          <t>EQ, NE, LIKE, ILIKE</t>
+          <t>EQ, NE</t>
         </is>
       </c>
     </row>
@@ -4993,7 +4993,7 @@
       </c>
       <c r="M145" t="inlineStr">
         <is>
-          <t>IS_NULL, EQ, NE, GT, GE, LT, LE, LIKE, ILIKE</t>
+          <t>IS_NULL, EQ, NE, GT, GE, LT, LE</t>
         </is>
       </c>
     </row>

</xml_diff>